<commit_message>
Terminologia: página do site vira "resumo prévio" e a nota técnica vira "parecer técnico"
- Site, painel, e-mails, carimbo dos PDFs, protótipos, modelos Word, guia da
  metodologia, planilha e documentação: o que o leitor vê passa a dizer
  "resumo prévio" (a página aberta) e "parecer técnico" (o PDF).
- Endereço da página: /resumos/<slug>; /pareceres e /pareceres/<slug>
  redirecionam de forma permanente (308).
- O sentido legislativo de "parecer" (parecer do relator, de comissão) e os
  nomes internos do código (coleção pareceres, campo notaTecnica) não mudam.
- modelo-nota-tecnica.docx passa a se chamar modelo-parecer-tecnico.docx.
- Teste da conta do inscrito: espera de até 15 s pelo salvamento em segundo plano.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019xgzxFHuUdfQmM6KHZGaMU
</commit_message>
<xml_diff>
--- a/docs/modelos/planilha-hipoteses-e-graficos.xlsx
+++ b/docs/modelos/planilha-hipoteses-e-graficos.xlsx
@@ -71,7 +71,7 @@
     <t xml:space="preserve">1. Preencha só as células amarelas (texto azul). As demais são fórmulas e se atualizam sozinhas.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Aba Hipóteses: uma linha por hipótese da nota técnica (parte 6). O critério sugere um resultado; o resultado final é sempre do autor (coluna L).</t>
+    <t xml:space="preserve">2. Aba Hipóteses: uma linha por hipótese do parecer técnico (parte 6). O critério sugere um resultado; o resultado final é sempre do autor (coluna L).</t>
   </si>
   <si>
     <t xml:space="preserve">3. Aba Cenários: valores do indicador da H1 por ano em cada cenário (A, B, C). O gráfico de trajetória e o limiar da H1 se atualizam.</t>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Nº</t>
   </si>
   <si>
-    <t xml:space="preserve">Hipótese (como na nota técnica)</t>
+    <t xml:space="preserve">Hipótese (como no parecer técnico)</t>
   </si>
   <si>
     <t xml:space="preserve">Indicador</t>
@@ -290,7 +290,7 @@
     <t xml:space="preserve">−2 piora muito · −1 piora · 0 sem mudança · +1 melhora · +2 melhora muito</t>
   </si>
   <si>
-    <t xml:space="preserve">Dimensões fixas: ambiental, social, econômica, institucional e fiscal (as mesmas da nota técnica, parte 7).</t>
+    <t xml:space="preserve">Dimensões fixas: ambiental, social, econômica, institucional e fiscal (as mesmas do parecer técnico, parte 7).</t>
   </si>
 </sst>
 </file>
@@ -1124,11 +1124,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="83424725"/>
-        <c:axId val="2001771"/>
+        <c:axId val="92360505"/>
+        <c:axId val="89634206"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="83424725"/>
+        <c:axId val="92360505"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1160,7 +1160,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2001771"/>
+        <c:crossAx val="89634206"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1168,7 +1168,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2001771"/>
+        <c:axId val="89634206"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1244,7 +1244,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83424725"/>
+        <c:crossAx val="92360505"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1489,11 +1489,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="-5"/>
-        <c:axId val="48082974"/>
-        <c:axId val="12972756"/>
+        <c:axId val="89837350"/>
+        <c:axId val="42469991"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="48082974"/>
+        <c:axId val="89837350"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1525,7 +1525,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12972756"/>
+        <c:crossAx val="42469991"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1533,7 +1533,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12972756"/>
+        <c:axId val="42469991"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="2"/>
@@ -1611,7 +1611,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48082974"/>
+        <c:crossAx val="89837350"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>

</xml_diff>

<commit_message>
Exemplo didático: parecer técnico e quadro comparativo da Lei nº 15.190/2025
- Parecer técnico nº 001/2026 (exemplo) sobre os arts. 9º e 22 da Lei Geral do
  Licenciamento Ambiental, com texto base literal (Câmara/Legin, com os vetos
  derrubados e a Lei nº 15.300/2025), regime anterior (CONAMA 237/1997, Lei
  6.938/1981), hipóteses H1 a H3 testadas com dados reais (MapBiomas, SFB/Sicar),
  cenários por premissa, soluções, casos (PPCDAm, Moratória da Soja) e conclusão.
- Quadro comparativo e planilha preenchidos com os mesmos dados; gráficos com a
  série observada 2022-2025 e os cenários.
- Planilha: hipóteses de nível ("acima de", "abaixo de") além de variação.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019xgzxFHuUdfQmM6KHZGaMU
</commit_message>
<xml_diff>
--- a/docs/modelos/planilha-hipoteses-e-graficos.xlsx
+++ b/docs/modelos/planilha-hipoteses-e-graficos.xlsx
@@ -36,7 +36,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Em proporção: 10% = 0,10. Para hipótese de redução, informe o limiar como positivo e escolha "redução" no sentido.</t>
+          <t xml:space="preserve">Em proporção: 10% = 0,10. Aumento/redução: o limiar é uma variação (para redução, informe positivo). Acima de/abaixo de: o limiar é um nível (ex.: 0,80 = 80%).</t>
         </r>
       </text>
     </comment>
@@ -131,10 +131,10 @@
     <t xml:space="preserve">Sentido esperado</t>
   </si>
   <si>
-    <t xml:space="preserve">Limiar (variação que sustenta a hipótese)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variação observada ou projetada</t>
+    <t xml:space="preserve">Limiar (variação ou nível que sustenta a hipótese)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observado (variação ou nível)</t>
   </si>
   <si>
     <t xml:space="preserve">Confiança da evidência</t>
@@ -297,11 +297,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
-    <numFmt numFmtId="166" formatCode="0%"/>
-    <numFmt numFmtId="167" formatCode="\+0;\-0;0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0%"/>
+    <numFmt numFmtId="168" formatCode="\+0;\-0;0"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -572,7 +573,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -580,7 +581,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1124,11 +1125,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="92360505"/>
-        <c:axId val="89634206"/>
+        <c:axId val="75561645"/>
+        <c:axId val="44954145"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="92360505"/>
+        <c:axId val="75561645"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1160,7 +1161,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89634206"/>
+        <c:crossAx val="44954145"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1168,7 +1169,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89634206"/>
+        <c:axId val="44954145"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1244,7 +1245,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92360505"/>
+        <c:crossAx val="75561645"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1489,11 +1490,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="-5"/>
-        <c:axId val="89837350"/>
-        <c:axId val="42469991"/>
+        <c:axId val="57248324"/>
+        <c:axId val="53243054"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="89837350"/>
+        <c:axId val="57248324"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1525,7 +1526,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42469991"/>
+        <c:crossAx val="53243054"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1533,7 +1534,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42469991"/>
+        <c:axId val="53243054"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="2"/>
@@ -1611,7 +1612,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89837350"/>
+        <c:crossAx val="57248324"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -2122,7 +2123,7 @@
         <v>36</v>
       </c>
       <c r="K2" s="15" t="str">
-        <f aca="false">IF(OR(H2="",I2=""),"Inconclusiva",IF(IF(G2="redução",-I2,I2)&gt;=ABS(H2),IF(J2="baixa","Sustentada em parte","Sustentada"),IF(IF(G2="redução",-I2,I2)&gt;=ABS(H2)/2,"Sustentada em parte","Não sustentada")))</f>
+        <f aca="false">IF(OR(H2="",I2=""),"Inconclusiva",IF(OR(AND(G2="aumento",I2&gt;=ABS(H2)),AND(G2="redução",-I2&gt;=ABS(H2)),AND(G2="acima de",I2&gt;=H2),AND(G2="abaixo de",I2&lt;=H2)),IF(J2="baixa","Sustentada em parte","Sustentada"),IF(OR(AND(G2="aumento",I2&gt;=ABS(H2)/2),AND(G2="redução",-I2&gt;=ABS(H2)/2)),"Sustentada em parte","Não sustentada")))</f>
         <v>Sustentada em parte</v>
       </c>
       <c r="L2" s="10" t="s">
@@ -2162,7 +2163,7 @@
         <v>36</v>
       </c>
       <c r="K3" s="15" t="str">
-        <f aca="false">IF(OR(H3="",I3=""),"Inconclusiva",IF(IF(G3="redução",-I3,I3)&gt;=ABS(H3),IF(J3="baixa","Sustentada em parte","Sustentada"),IF(IF(G3="redução",-I3,I3)&gt;=ABS(H3)/2,"Sustentada em parte","Não sustentada")))</f>
+        <f aca="false">IF(OR(H3="",I3=""),"Inconclusiva",IF(OR(AND(G3="aumento",I3&gt;=ABS(H3)),AND(G3="redução",-I3&gt;=ABS(H3)),AND(G3="acima de",I3&gt;=H3),AND(G3="abaixo de",I3&lt;=H3)),IF(J3="baixa","Sustentada em parte","Sustentada"),IF(OR(AND(G3="aumento",I3&gt;=ABS(H3)/2),AND(G3="redução",-I3&gt;=ABS(H3)/2)),"Sustentada em parte","Não sustentada")))</f>
         <v>Inconclusiva</v>
       </c>
       <c r="L3" s="10"/>
@@ -2184,7 +2185,7 @@
       <c r="I4" s="14"/>
       <c r="J4" s="10"/>
       <c r="K4" s="15" t="str">
-        <f aca="false">IF(OR(H4="",I4=""),"Inconclusiva",IF(IF(G4="redução",-I4,I4)&gt;=ABS(H4),IF(J4="baixa","Sustentada em parte","Sustentada"),IF(IF(G4="redução",-I4,I4)&gt;=ABS(H4)/2,"Sustentada em parte","Não sustentada")))</f>
+        <f aca="false">IF(OR(H4="",I4=""),"Inconclusiva",IF(OR(AND(G4="aumento",I4&gt;=ABS(H4)),AND(G4="redução",-I4&gt;=ABS(H4)),AND(G4="acima de",I4&gt;=H4),AND(G4="abaixo de",I4&lt;=H4)),IF(J4="baixa","Sustentada em parte","Sustentada"),IF(OR(AND(G4="aumento",I4&gt;=ABS(H4)/2),AND(G4="redução",-I4&gt;=ABS(H4)/2)),"Sustentada em parte","Não sustentada")))</f>
         <v>Inconclusiva</v>
       </c>
       <c r="L4" s="10"/>
@@ -2204,7 +2205,7 @@
       <c r="I5" s="14"/>
       <c r="J5" s="10"/>
       <c r="K5" s="15" t="str">
-        <f aca="false">IF(OR(H5="",I5=""),"Inconclusiva",IF(IF(G5="redução",-I5,I5)&gt;=ABS(H5),IF(J5="baixa","Sustentada em parte","Sustentada"),IF(IF(G5="redução",-I5,I5)&gt;=ABS(H5)/2,"Sustentada em parte","Não sustentada")))</f>
+        <f aca="false">IF(OR(H5="",I5=""),"Inconclusiva",IF(OR(AND(G5="aumento",I5&gt;=ABS(H5)),AND(G5="redução",-I5&gt;=ABS(H5)),AND(G5="acima de",I5&gt;=H5),AND(G5="abaixo de",I5&lt;=H5)),IF(J5="baixa","Sustentada em parte","Sustentada"),IF(OR(AND(G5="aumento",I5&gt;=ABS(H5)/2),AND(G5="redução",-I5&gt;=ABS(H5)/2)),"Sustentada em parte","Não sustentada")))</f>
         <v>Inconclusiva</v>
       </c>
       <c r="L5" s="10"/>
@@ -2224,7 +2225,7 @@
       <c r="I6" s="14"/>
       <c r="J6" s="10"/>
       <c r="K6" s="15" t="str">
-        <f aca="false">IF(OR(H6="",I6=""),"Inconclusiva",IF(IF(G6="redução",-I6,I6)&gt;=ABS(H6),IF(J6="baixa","Sustentada em parte","Sustentada"),IF(IF(G6="redução",-I6,I6)&gt;=ABS(H6)/2,"Sustentada em parte","Não sustentada")))</f>
+        <f aca="false">IF(OR(H6="",I6=""),"Inconclusiva",IF(OR(AND(G6="aumento",I6&gt;=ABS(H6)),AND(G6="redução",-I6&gt;=ABS(H6)),AND(G6="acima de",I6&gt;=H6),AND(G6="abaixo de",I6&lt;=H6)),IF(J6="baixa","Sustentada em parte","Sustentada"),IF(OR(AND(G6="aumento",I6&gt;=ABS(H6)/2),AND(G6="redução",-I6&gt;=ABS(H6)/2)),"Sustentada em parte","Não sustentada")))</f>
         <v>Inconclusiva</v>
       </c>
       <c r="L6" s="10"/>
@@ -2244,7 +2245,7 @@
       <c r="I7" s="14"/>
       <c r="J7" s="10"/>
       <c r="K7" s="15" t="str">
-        <f aca="false">IF(OR(H7="",I7=""),"Inconclusiva",IF(IF(G7="redução",-I7,I7)&gt;=ABS(H7),IF(J7="baixa","Sustentada em parte","Sustentada"),IF(IF(G7="redução",-I7,I7)&gt;=ABS(H7)/2,"Sustentada em parte","Não sustentada")))</f>
+        <f aca="false">IF(OR(H7="",I7=""),"Inconclusiva",IF(OR(AND(G7="aumento",I7&gt;=ABS(H7)),AND(G7="redução",-I7&gt;=ABS(H7)),AND(G7="acima de",I7&gt;=H7),AND(G7="abaixo de",I7&lt;=H7)),IF(J7="baixa","Sustentada em parte","Sustentada"),IF(OR(AND(G7="aumento",I7&gt;=ABS(H7)/2),AND(G7="redução",-I7&gt;=ABS(H7)/2)),"Sustentada em parte","Não sustentada")))</f>
         <v>Inconclusiva</v>
       </c>
       <c r="L7" s="10"/>
@@ -2278,7 +2279,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G7" type="list">
-      <formula1>"aumento,redução"</formula1>
+      <formula1>"aumento,redução,acima de,abaixo de"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J7" type="list">

</xml_diff>